<commit_message>
Updated to xlsx download files for local data
</commit_message>
<xml_diff>
--- a/datasets/local-data/FoE-local-env-data-MAYORAL-2026.xlsx
+++ b/datasets/local-data/FoE-local-env-data-MAYORAL-2026.xlsx
@@ -158,19 +158,19 @@
     <t xml:space="preserve">Greenspace: m2 perpop tertile</t>
   </si>
   <si>
+    <t xml:space="preserve">Flooding (England): current high risk properties</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flooding (England): future high risk properties</t>
+  </si>
+  <si>
     <t xml:space="preserve">Flooding (England): current high risk people</t>
   </si>
   <si>
-    <t xml:space="preserve">Flooding (England): current high risk properties</t>
-  </si>
-  <si>
     <t xml:space="preserve">Flooding (England): current high risk homes</t>
   </si>
   <si>
     <t xml:space="preserve">Flooding (England): future high risk people</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flooding (England): future high risk properties</t>
   </si>
   <si>
     <t xml:space="preserve">Flooding (England): future high risk homes</t>
@@ -1278,19 +1278,19 @@
         <v>88</v>
       </c>
       <c r="AW2" s="5" t="n">
+        <v>53290</v>
+      </c>
+      <c r="AX2" s="5" t="n">
+        <v>116470</v>
+      </c>
+      <c r="AY2" s="5" t="n">
         <v>78010</v>
       </c>
-      <c r="AX2" s="5" t="n">
-        <v>53290</v>
-      </c>
-      <c r="AY2" s="5" t="n">
+      <c r="AZ2" s="5" t="n">
         <v>33840</v>
       </c>
-      <c r="AZ2" s="5" t="n">
+      <c r="BA2" s="5" t="n">
         <v>163610</v>
-      </c>
-      <c r="BA2" s="5" t="n">
-        <v>116470</v>
       </c>
       <c r="BB2" s="5" t="n">
         <v>71060</v>
@@ -1484,7 +1484,7 @@
         <v>0.39</v>
       </c>
       <c r="AF3" s="5" t="n">
-        <v>36740</v>
+        <v>36750</v>
       </c>
       <c r="AG3" s="5" t="n">
         <v>6354</v>
@@ -1535,19 +1535,19 @@
         <v>92</v>
       </c>
       <c r="AW3" s="5" t="n">
+        <v>25860</v>
+      </c>
+      <c r="AX3" s="5" t="n">
+        <v>54670</v>
+      </c>
+      <c r="AY3" s="5" t="n">
         <v>34460</v>
       </c>
-      <c r="AX3" s="5" t="n">
-        <v>25860</v>
-      </c>
-      <c r="AY3" s="5" t="n">
+      <c r="AZ3" s="5" t="n">
         <v>14840</v>
       </c>
-      <c r="AZ3" s="5" t="n">
+      <c r="BA3" s="5" t="n">
         <v>74090</v>
-      </c>
-      <c r="BA3" s="5" t="n">
-        <v>54670</v>
       </c>
       <c r="BB3" s="5" t="n">
         <v>32750</v>
@@ -1741,7 +1741,7 @@
         <v>0.56</v>
       </c>
       <c r="AF4" s="5" t="n">
-        <v>44300</v>
+        <v>44290</v>
       </c>
       <c r="AG4" s="5" t="n">
         <v>8865</v>
@@ -1792,19 +1792,19 @@
         <v>95</v>
       </c>
       <c r="AW4" s="5" t="n">
+        <v>47490</v>
+      </c>
+      <c r="AX4" s="5" t="n">
+        <v>88950</v>
+      </c>
+      <c r="AY4" s="5" t="n">
         <v>53140</v>
       </c>
-      <c r="AX4" s="5" t="n">
-        <v>47490</v>
-      </c>
-      <c r="AY4" s="5" t="n">
+      <c r="AZ4" s="5" t="n">
         <v>23590</v>
       </c>
-      <c r="AZ4" s="5" t="n">
+      <c r="BA4" s="5" t="n">
         <v>102090</v>
-      </c>
-      <c r="BA4" s="5" t="n">
-        <v>88950</v>
       </c>
       <c r="BB4" s="5" t="n">
         <v>45450</v>
@@ -1998,7 +1998,7 @@
         <v>0.56</v>
       </c>
       <c r="AF5" s="5" t="n">
-        <v>28860</v>
+        <v>28870</v>
       </c>
       <c r="AG5" s="5" t="n">
         <v>3222</v>
@@ -2049,19 +2049,19 @@
         <v>88</v>
       </c>
       <c r="AW5" s="5" t="n">
+        <v>58020</v>
+      </c>
+      <c r="AX5" s="5" t="n">
+        <v>92650</v>
+      </c>
+      <c r="AY5" s="5" t="n">
         <v>87860</v>
       </c>
-      <c r="AX5" s="5" t="n">
-        <v>58020</v>
-      </c>
-      <c r="AY5" s="5" t="n">
+      <c r="AZ5" s="5" t="n">
         <v>39590</v>
       </c>
-      <c r="AZ5" s="5" t="n">
+      <c r="BA5" s="5" t="n">
         <v>138050</v>
-      </c>
-      <c r="BA5" s="5" t="n">
-        <v>92650</v>
       </c>
       <c r="BB5" s="5" t="n">
         <v>62930</v>
@@ -2255,7 +2255,7 @@
         <v>0.21</v>
       </c>
       <c r="AF6" s="5" t="n">
-        <v>17770</v>
+        <v>17760</v>
       </c>
       <c r="AG6" s="5" t="n">
         <v>3402</v>
@@ -2306,19 +2306,19 @@
         <v>95</v>
       </c>
       <c r="AW6" s="5" t="n">
+        <v>18390</v>
+      </c>
+      <c r="AX6" s="5" t="n">
+        <v>35240</v>
+      </c>
+      <c r="AY6" s="5" t="n">
         <v>26930</v>
       </c>
-      <c r="AX6" s="5" t="n">
-        <v>18390</v>
-      </c>
-      <c r="AY6" s="5" t="n">
+      <c r="AZ6" s="5" t="n">
         <v>12270</v>
       </c>
-      <c r="AZ6" s="5" t="n">
+      <c r="BA6" s="5" t="n">
         <v>51720</v>
-      </c>
-      <c r="BA6" s="5" t="n">
-        <v>35240</v>
       </c>
       <c r="BB6" s="5" t="n">
         <v>23670</v>
@@ -2563,19 +2563,19 @@
         <v>88</v>
       </c>
       <c r="AW7" s="5" t="n">
+        <v>45880</v>
+      </c>
+      <c r="AX7" s="5" t="n">
+        <v>98750</v>
+      </c>
+      <c r="AY7" s="5" t="n">
         <v>74990</v>
       </c>
-      <c r="AX7" s="5" t="n">
-        <v>45880</v>
-      </c>
-      <c r="AY7" s="5" t="n">
+      <c r="AZ7" s="5" t="n">
         <v>29780</v>
       </c>
-      <c r="AZ7" s="5" t="n">
+      <c r="BA7" s="5" t="n">
         <v>158700</v>
-      </c>
-      <c r="BA7" s="5" t="n">
-        <v>98750</v>
       </c>
       <c r="BB7" s="5" t="n">
         <v>62690</v>
@@ -2769,7 +2769,7 @@
         <v>0.43</v>
       </c>
       <c r="AF8" s="5" t="n">
-        <v>42190</v>
+        <v>42180</v>
       </c>
       <c r="AG8" s="5" t="n">
         <v>19712</v>
@@ -2820,19 +2820,19 @@
         <v>88</v>
       </c>
       <c r="AW8" s="5" t="n">
+        <v>33910</v>
+      </c>
+      <c r="AX8" s="5" t="n">
+        <v>79050</v>
+      </c>
+      <c r="AY8" s="5" t="n">
         <v>45620</v>
       </c>
-      <c r="AX8" s="5" t="n">
-        <v>33910</v>
-      </c>
-      <c r="AY8" s="5" t="n">
+      <c r="AZ8" s="5" t="n">
         <v>18960</v>
       </c>
-      <c r="AZ8" s="5" t="n">
+      <c r="BA8" s="5" t="n">
         <v>107250</v>
-      </c>
-      <c r="BA8" s="5" t="n">
-        <v>79050</v>
       </c>
       <c r="BB8" s="5" t="n">
         <v>44460</v>
@@ -3026,7 +3026,7 @@
         <v>0.51</v>
       </c>
       <c r="AF9" s="5" t="n">
-        <v>23620</v>
+        <v>23630</v>
       </c>
       <c r="AG9" s="5" t="n">
         <v>8225</v>
@@ -3077,19 +3077,19 @@
         <v>88</v>
       </c>
       <c r="AW9" s="5" t="n">
+        <v>37040</v>
+      </c>
+      <c r="AX9" s="5" t="n">
+        <v>65950</v>
+      </c>
+      <c r="AY9" s="5" t="n">
         <v>55040</v>
       </c>
-      <c r="AX9" s="5" t="n">
-        <v>37040</v>
-      </c>
-      <c r="AY9" s="5" t="n">
+      <c r="AZ9" s="5" t="n">
         <v>22970</v>
       </c>
-      <c r="AZ9" s="5" t="n">
+      <c r="BA9" s="5" t="n">
         <v>98500</v>
-      </c>
-      <c r="BA9" s="5" t="n">
-        <v>65950</v>
       </c>
       <c r="BB9" s="5" t="n">
         <v>41840</v>
@@ -3332,19 +3332,19 @@
         <v>92</v>
       </c>
       <c r="AW10" s="5" t="n">
+        <v>32790</v>
+      </c>
+      <c r="AX10" s="5" t="n">
+        <v>58630</v>
+      </c>
+      <c r="AY10" s="5" t="n">
         <v>34000</v>
       </c>
-      <c r="AX10" s="5" t="n">
-        <v>32790</v>
-      </c>
-      <c r="AY10" s="5" t="n">
+      <c r="AZ10" s="5" t="n">
         <v>14880</v>
       </c>
-      <c r="AZ10" s="5" t="n">
+      <c r="BA10" s="5" t="n">
         <v>64850</v>
-      </c>
-      <c r="BA10" s="5" t="n">
-        <v>58630</v>
       </c>
       <c r="BB10" s="5" t="n">
         <v>28640</v>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="AE11" s="5"/>
       <c r="AF11" s="5" t="n">
-        <v>66980</v>
+        <v>66950</v>
       </c>
       <c r="AG11" s="5" t="n">
         <v>15323</v>
@@ -3587,19 +3587,19 @@
         <v>92</v>
       </c>
       <c r="AW11" s="5" t="n">
+        <v>49440</v>
+      </c>
+      <c r="AX11" s="5" t="n">
+        <v>100590</v>
+      </c>
+      <c r="AY11" s="5" t="n">
         <v>61540</v>
       </c>
-      <c r="AX11" s="5" t="n">
-        <v>49440</v>
-      </c>
-      <c r="AY11" s="5" t="n">
+      <c r="AZ11" s="5" t="n">
         <v>26410</v>
       </c>
-      <c r="AZ11" s="5" t="n">
+      <c r="BA11" s="5" t="n">
         <v>129780</v>
-      </c>
-      <c r="BA11" s="5" t="n">
-        <v>100590</v>
       </c>
       <c r="BB11" s="5" t="n">
         <v>56690</v>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="AE12" s="5"/>
       <c r="AF12" s="5" t="n">
-        <v>60020</v>
+        <v>60030</v>
       </c>
       <c r="AG12" s="5" t="n">
         <v>11485</v>
@@ -3842,19 +3842,19 @@
         <v>92</v>
       </c>
       <c r="AW12" s="5" t="n">
+        <v>41700</v>
+      </c>
+      <c r="AX12" s="5" t="n">
+        <v>73700</v>
+      </c>
+      <c r="AY12" s="5" t="n">
         <v>52650</v>
       </c>
-      <c r="AX12" s="5" t="n">
-        <v>41700</v>
-      </c>
-      <c r="AY12" s="5" t="n">
+      <c r="AZ12" s="5" t="n">
         <v>23700</v>
       </c>
-      <c r="AZ12" s="5" t="n">
+      <c r="BA12" s="5" t="n">
         <v>96590</v>
-      </c>
-      <c r="BA12" s="5" t="n">
-        <v>73700</v>
       </c>
       <c r="BB12" s="5" t="n">
         <v>44330</v>
@@ -4097,19 +4097,19 @@
         <v>95</v>
       </c>
       <c r="AW13" s="5" t="n">
+        <v>31200</v>
+      </c>
+      <c r="AX13" s="5" t="n">
+        <v>48310</v>
+      </c>
+      <c r="AY13" s="5" t="n">
         <v>41670</v>
       </c>
-      <c r="AX13" s="5" t="n">
-        <v>31200</v>
-      </c>
-      <c r="AY13" s="5" t="n">
+      <c r="AZ13" s="5" t="n">
         <v>18430</v>
       </c>
-      <c r="AZ13" s="5" t="n">
+      <c r="BA13" s="5" t="n">
         <v>62720</v>
-      </c>
-      <c r="BA13" s="5" t="n">
-        <v>48310</v>
       </c>
       <c r="BB13" s="5" t="n">
         <v>28190</v>
@@ -4352,19 +4352,19 @@
         <v>95</v>
       </c>
       <c r="AW14" s="5" t="n">
+        <v>76070</v>
+      </c>
+      <c r="AX14" s="5" t="n">
+        <v>139510</v>
+      </c>
+      <c r="AY14" s="5" t="n">
         <v>64400</v>
       </c>
-      <c r="AX14" s="5" t="n">
-        <v>76070</v>
-      </c>
-      <c r="AY14" s="5" t="n">
+      <c r="AZ14" s="5" t="n">
         <v>29440</v>
       </c>
-      <c r="AZ14" s="5" t="n">
+      <c r="BA14" s="5" t="n">
         <v>152940</v>
-      </c>
-      <c r="BA14" s="5" t="n">
-        <v>139510</v>
       </c>
       <c r="BB14" s="5" t="n">
         <v>67890</v>
@@ -4607,19 +4607,19 @@
         <v>92</v>
       </c>
       <c r="AW15" s="5" t="n">
+        <v>21120</v>
+      </c>
+      <c r="AX15" s="5" t="n">
+        <v>33100</v>
+      </c>
+      <c r="AY15" s="5" t="n">
         <v>21430</v>
       </c>
-      <c r="AX15" s="5" t="n">
-        <v>21120</v>
-      </c>
-      <c r="AY15" s="5" t="n">
+      <c r="AZ15" s="5" t="n">
         <v>9860</v>
       </c>
-      <c r="AZ15" s="5" t="n">
+      <c r="BA15" s="5" t="n">
         <v>34430</v>
-      </c>
-      <c r="BA15" s="5" t="n">
-        <v>33100</v>
       </c>
       <c r="BB15" s="5" t="n">
         <v>16090</v>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="AE16" s="5"/>
       <c r="AF16" s="5" t="n">
-        <v>26860</v>
+        <v>26870</v>
       </c>
       <c r="AG16" s="5" t="n">
         <v>7005</v>
@@ -4862,19 +4862,19 @@
         <v>95</v>
       </c>
       <c r="AW16" s="5" t="n">
+        <v>26240</v>
+      </c>
+      <c r="AX16" s="5" t="n">
+        <v>45600</v>
+      </c>
+      <c r="AY16" s="5" t="n">
         <v>29940</v>
       </c>
-      <c r="AX16" s="5" t="n">
-        <v>26240</v>
-      </c>
-      <c r="AY16" s="5" t="n">
+      <c r="AZ16" s="5" t="n">
         <v>13070</v>
       </c>
-      <c r="AZ16" s="5" t="n">
+      <c r="BA16" s="5" t="n">
         <v>57820</v>
-      </c>
-      <c r="BA16" s="5" t="n">
-        <v>45600</v>
       </c>
       <c r="BB16" s="5" t="n">
         <v>25480</v>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="AE17" s="5"/>
       <c r="AF17" s="5" t="n">
-        <v>47260</v>
+        <v>47280</v>
       </c>
       <c r="AG17" s="5" t="n">
         <v>21500</v>
@@ -5117,19 +5117,19 @@
         <v>95</v>
       </c>
       <c r="AW17" s="5" t="n">
+        <v>102500</v>
+      </c>
+      <c r="AX17" s="5" t="n">
+        <v>143200</v>
+      </c>
+      <c r="AY17" s="5" t="n">
         <v>158300</v>
       </c>
-      <c r="AX17" s="5" t="n">
-        <v>102500</v>
-      </c>
-      <c r="AY17" s="5" t="n">
+      <c r="AZ17" s="5" t="n">
         <v>64290</v>
       </c>
-      <c r="AZ17" s="5" t="n">
+      <c r="BA17" s="5" t="n">
         <v>218470</v>
-      </c>
-      <c r="BA17" s="5" t="n">
-        <v>143200</v>
       </c>
       <c r="BB17" s="5" t="n">
         <v>90310</v>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="AE18" s="5"/>
       <c r="AF18" s="5" t="n">
-        <v>60810</v>
+        <v>60820</v>
       </c>
       <c r="AG18" s="5" t="n">
         <v>20376</v>
@@ -5372,19 +5372,19 @@
         <v>92</v>
       </c>
       <c r="AW18" s="5" t="n">
+        <v>39010</v>
+      </c>
+      <c r="AX18" s="5" t="n">
+        <v>66100</v>
+      </c>
+      <c r="AY18" s="5" t="n">
         <v>51720</v>
       </c>
-      <c r="AX18" s="5" t="n">
-        <v>39010</v>
-      </c>
-      <c r="AY18" s="5" t="n">
+      <c r="AZ18" s="5" t="n">
         <v>22680</v>
       </c>
-      <c r="AZ18" s="5" t="n">
+      <c r="BA18" s="5" t="n">
         <v>90860</v>
-      </c>
-      <c r="BA18" s="5" t="n">
-        <v>66100</v>
       </c>
       <c r="BB18" s="5" t="n">
         <v>40000</v>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="AE19" s="5"/>
       <c r="AF19" s="5" t="n">
-        <v>75050</v>
+        <v>75040</v>
       </c>
       <c r="AG19" s="5" t="n">
         <v>61244</v>
@@ -5627,19 +5627,19 @@
         <v>92</v>
       </c>
       <c r="AW19" s="5" t="n">
+        <v>69500</v>
+      </c>
+      <c r="AX19" s="5" t="n">
+        <v>116000</v>
+      </c>
+      <c r="AY19" s="5" t="n">
         <v>74050</v>
       </c>
-      <c r="AX19" s="5" t="n">
-        <v>69500</v>
-      </c>
-      <c r="AY19" s="5" t="n">
+      <c r="AZ19" s="5" t="n">
         <v>33270</v>
       </c>
-      <c r="AZ19" s="5" t="n">
+      <c r="BA19" s="5" t="n">
         <v>130120</v>
-      </c>
-      <c r="BA19" s="5" t="n">
-        <v>116000</v>
       </c>
       <c r="BB19" s="5" t="n">
         <v>58110</v>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="AE20" s="5"/>
       <c r="AF20" s="5" t="n">
-        <v>48080</v>
+        <v>48090</v>
       </c>
       <c r="AG20" s="5" t="n">
         <v>18229</v>
@@ -5882,19 +5882,19 @@
         <v>95</v>
       </c>
       <c r="AW20" s="5" t="n">
+        <v>61870</v>
+      </c>
+      <c r="AX20" s="5" t="n">
+        <v>95380</v>
+      </c>
+      <c r="AY20" s="5" t="n">
         <v>70030</v>
       </c>
-      <c r="AX20" s="5" t="n">
-        <v>61870</v>
-      </c>
-      <c r="AY20" s="5" t="n">
+      <c r="AZ20" s="5" t="n">
         <v>32380</v>
       </c>
-      <c r="AZ20" s="5" t="n">
+      <c r="BA20" s="5" t="n">
         <v>112490</v>
-      </c>
-      <c r="BA20" s="5" t="n">
-        <v>95380</v>
       </c>
       <c r="BB20" s="5" t="n">
         <v>51750</v>
@@ -6088,7 +6088,7 @@
         <v>0.66</v>
       </c>
       <c r="AF21" s="7" t="n">
-        <v>64070</v>
+        <v>64060</v>
       </c>
       <c r="AG21" s="7" t="n">
         <v>47984</v>
@@ -6139,19 +6139,19 @@
         <v>88</v>
       </c>
       <c r="AW21" s="7" t="n">
+        <v>433800</v>
+      </c>
+      <c r="AX21" s="7" t="n">
+        <v>727630</v>
+      </c>
+      <c r="AY21" s="7" t="n">
         <v>626480</v>
       </c>
-      <c r="AX21" s="7" t="n">
-        <v>433800</v>
-      </c>
-      <c r="AY21" s="7" t="n">
+      <c r="AZ21" s="7" t="n">
         <v>257810</v>
       </c>
-      <c r="AZ21" s="7" t="n">
+      <c r="BA21" s="7" t="n">
         <v>1079790</v>
-      </c>
-      <c r="BA21" s="7" t="n">
-        <v>727630</v>
       </c>
       <c r="BB21" s="7" t="n">
         <v>439950</v>

</xml_diff>